<commit_message>
Bộ file gửi thẳng cho người dùng, chỉnh số luồng trong config.txt
- Thêm 2 file .bat bấm đúp là chạy, và file DOC FILE NAY TRUOC.txt
  hướng dẫn 4 bước
- Số ảnh chạy cùng lúc đặt được trong config.txt, không cần dòng
  lệnh. Trần hạ từ 10 xuống 5.
- Lưu API key không còn ghi đè cả file, giữ nguyên cài đặt người
  dùng đã sửa
- Bỏ đường dẫn ảnh giả trong file mẫu: chạy lần đầu báo "không tìm
  thấy ảnh" làm người mới tưởng mình làm sai
- File .bat gọi exe bằng đường dẫn tuyệt đối, không phụ thuộc thư
  mục hiện tại
- Chỉ dẫn liên hệ nhận quota dùng thử ở chỗ hỏi API key
- Bỏ mục ghi chú API khỏi README

81 test.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mau.xlsx
+++ b/mau.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Danh sach anh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sach anh" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,14 +535,10 @@
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A cozy bookshop interior in autumn, warm lamp light, wooden shelves full of books, rain on the window, painted in the same art style as the reference</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>D:\anh\phong-cach.jpg</t>
-        </is>
-      </c>
+          <t>A cozy bookshop interior in autumn, warm lamp light, wooden shelves full of books, rain on the window, soft painterly style</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>16:9</t>
@@ -557,14 +553,10 @@
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Banner for a coffee brand, the logo from the reference placed top-left, roasted beans scattered on dark wood, dramatic side lighting, copy space right</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>D:\anh\logo.png; https://example.com/anh-mau.jpg</t>
-        </is>
-      </c>
+          <t>Banner for a coffee brand, roasted beans scattered on dark wood, dramatic side lighting, generous copy space on the right</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>16:9</t>

</xml_diff>